<commit_message>
data: Actualización automática de reportes (2026-08-21 12:32)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
+++ b/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/VENTAS_MENSUALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDEF47C-2F0A-224E-916B-5B22425C2045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3626C529-91B5-C149-9FDB-4DBFC633F59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas Mensuales " sheetId="1" r:id="rId1"/>
@@ -928,11 +928,11 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1272,16 +1272,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -2184,16 +2184,16 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -3123,16 +3123,16 @@
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="1" t="s">
+      <c r="A94" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-      <c r="D94" s="1"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="1"/>
+      <c r="B94" s="5"/>
+      <c r="C94" s="5"/>
+      <c r="D94" s="5"/>
+      <c r="E94" s="5"/>
+      <c r="F94" s="5"/>
+      <c r="G94" s="5"/>
+      <c r="H94" s="5"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
@@ -4067,16 +4067,16 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A134" s="1" t="s">
+      <c r="A134" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B134" s="1"/>
-      <c r="C134" s="1"/>
-      <c r="D134" s="1"/>
-      <c r="E134" s="1"/>
-      <c r="F134" s="1"/>
-      <c r="G134" s="1"/>
-      <c r="H134" s="1"/>
+      <c r="B134" s="5"/>
+      <c r="C134" s="5"/>
+      <c r="D134" s="5"/>
+      <c r="E134" s="5"/>
+      <c r="F134" s="5"/>
+      <c r="G134" s="5"/>
+      <c r="H134" s="5"/>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
@@ -4352,7 +4352,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I144" s="1" t="s">
+      <c r="I144" s="5" t="s">
         <v>69</v>
       </c>
       <c r="K144" t="s">
@@ -4377,7 +4377,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I145" s="1"/>
+      <c r="I145" s="5"/>
       <c r="K145" t="s">
         <v>66</v>
       </c>
@@ -4406,7 +4406,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I146" s="1"/>
+      <c r="I146" s="5"/>
       <c r="K146" t="s">
         <v>75</v>
       </c>
@@ -4435,7 +4435,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I147" s="1"/>
+      <c r="I147" s="5"/>
       <c r="K147" t="s">
         <v>79</v>
       </c>
@@ -4928,16 +4928,16 @@
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A172" s="1" t="s">
+      <c r="A172" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B172" s="1"/>
-      <c r="C172" s="1"/>
-      <c r="D172" s="1"/>
-      <c r="E172" s="1"/>
-      <c r="F172" s="1"/>
-      <c r="G172" s="1"/>
-      <c r="H172" s="1"/>
+      <c r="B172" s="5"/>
+      <c r="C172" s="5"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+      <c r="F172" s="5"/>
+      <c r="G172" s="5"/>
+      <c r="H172" s="5"/>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
@@ -5760,16 +5760,16 @@
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A212" s="1" t="s">
+      <c r="A212" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B212" s="1"/>
-      <c r="C212" s="1"/>
-      <c r="D212" s="1"/>
-      <c r="E212" s="1"/>
-      <c r="F212" s="1"/>
-      <c r="G212" s="1"/>
-      <c r="H212" s="1"/>
+      <c r="B212" s="5"/>
+      <c r="C212" s="5"/>
+      <c r="D212" s="5"/>
+      <c r="E212" s="5"/>
+      <c r="F212" s="5"/>
+      <c r="G212" s="5"/>
+      <c r="H212" s="5"/>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
@@ -6607,16 +6607,16 @@
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A254" s="1" t="s">
+      <c r="A254" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B254" s="1"/>
-      <c r="C254" s="1"/>
-      <c r="D254" s="1"/>
-      <c r="E254" s="1"/>
-      <c r="F254" s="1"/>
-      <c r="G254" s="1"/>
-      <c r="H254" s="1"/>
+      <c r="B254" s="5"/>
+      <c r="C254" s="5"/>
+      <c r="D254" s="5"/>
+      <c r="E254" s="5"/>
+      <c r="F254" s="5"/>
+      <c r="G254" s="5"/>
+      <c r="H254" s="5"/>
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
@@ -7542,16 +7542,16 @@
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A302" s="1" t="s">
+      <c r="A302" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B302" s="1"/>
-      <c r="C302" s="1"/>
-      <c r="D302" s="1"/>
-      <c r="E302" s="1"/>
-      <c r="F302" s="1"/>
-      <c r="G302" s="1"/>
-      <c r="H302" s="1"/>
+      <c r="B302" s="5"/>
+      <c r="C302" s="5"/>
+      <c r="D302" s="5"/>
+      <c r="E302" s="5"/>
+      <c r="F302" s="5"/>
+      <c r="G302" s="5"/>
+      <c r="H302" s="5"/>
     </row>
     <row r="303" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
@@ -8547,16 +8547,16 @@
       </c>
     </row>
     <row r="353" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A353" s="1" t="s">
+      <c r="A353" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B353" s="1"/>
-      <c r="C353" s="1"/>
-      <c r="D353" s="1"/>
-      <c r="E353" s="1"/>
-      <c r="F353" s="1"/>
-      <c r="G353" s="1"/>
-      <c r="H353" s="1"/>
+      <c r="B353" s="5"/>
+      <c r="C353" s="5"/>
+      <c r="D353" s="5"/>
+      <c r="E353" s="5"/>
+      <c r="F353" s="5"/>
+      <c r="G353" s="5"/>
+      <c r="H353" s="5"/>
     </row>
     <row r="354" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
@@ -9615,16 +9615,16 @@
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A411" s="1" t="s">
+      <c r="A411" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="B411" s="1"/>
-      <c r="C411" s="1"/>
-      <c r="D411" s="1"/>
-      <c r="E411" s="1"/>
-      <c r="F411" s="1"/>
-      <c r="G411" s="1"/>
-      <c r="H411" s="1"/>
+      <c r="B411" s="5"/>
+      <c r="C411" s="5"/>
+      <c r="D411" s="5"/>
+      <c r="E411" s="5"/>
+      <c r="F411" s="5"/>
+      <c r="G411" s="5"/>
+      <c r="H411" s="5"/>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
@@ -10718,16 +10718,16 @@
       </c>
     </row>
     <row r="463" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A463" s="1" t="s">
+      <c r="A463" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B463" s="1"/>
-      <c r="C463" s="1"/>
-      <c r="D463" s="1"/>
-      <c r="E463" s="1"/>
-      <c r="F463" s="1"/>
-      <c r="G463" s="1"/>
-      <c r="H463" s="1"/>
+      <c r="B463" s="5"/>
+      <c r="C463" s="5"/>
+      <c r="D463" s="5"/>
+      <c r="E463" s="5"/>
+      <c r="F463" s="5"/>
+      <c r="G463" s="5"/>
+      <c r="H463" s="5"/>
     </row>
     <row r="464" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
@@ -12032,16 +12032,16 @@
       </c>
     </row>
     <row r="528" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A528" s="1" t="s">
+      <c r="A528" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="B528" s="1"/>
-      <c r="C528" s="1"/>
-      <c r="D528" s="1"/>
-      <c r="E528" s="1"/>
-      <c r="F528" s="1"/>
-      <c r="G528" s="1"/>
-      <c r="H528" s="1"/>
+      <c r="B528" s="5"/>
+      <c r="C528" s="5"/>
+      <c r="D528" s="5"/>
+      <c r="E528" s="5"/>
+      <c r="F528" s="5"/>
+      <c r="G528" s="5"/>
+      <c r="H528" s="5"/>
     </row>
     <row r="529" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A529" t="s">
@@ -13365,16 +13365,16 @@
       </c>
     </row>
     <row r="585" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A585" s="1" t="s">
+      <c r="A585" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B585" s="1"/>
-      <c r="C585" s="1"/>
-      <c r="D585" s="1"/>
-      <c r="E585" s="1"/>
-      <c r="F585" s="1"/>
-      <c r="G585" s="1"/>
-      <c r="H585" s="1"/>
+      <c r="B585" s="5"/>
+      <c r="C585" s="5"/>
+      <c r="D585" s="5"/>
+      <c r="E585" s="5"/>
+      <c r="F585" s="5"/>
+      <c r="G585" s="5"/>
+      <c r="H585" s="5"/>
     </row>
     <row r="586" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
@@ -15052,16 +15052,16 @@
       </c>
     </row>
     <row r="667" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A667" s="1" t="s">
+      <c r="A667" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B667" s="1"/>
-      <c r="C667" s="1"/>
-      <c r="D667" s="1"/>
-      <c r="E667" s="1"/>
-      <c r="F667" s="1"/>
-      <c r="G667" s="1"/>
-      <c r="H667" s="1"/>
+      <c r="B667" s="5"/>
+      <c r="C667" s="5"/>
+      <c r="D667" s="5"/>
+      <c r="E667" s="5"/>
+      <c r="F667" s="5"/>
+      <c r="G667" s="5"/>
+      <c r="H667" s="5"/>
     </row>
     <row r="668" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A668" t="s">
@@ -16797,16 +16797,16 @@
       </c>
     </row>
     <row r="752" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A752" s="1" t="s">
+      <c r="A752" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B752" s="1"/>
-      <c r="C752" s="1"/>
-      <c r="D752" s="1"/>
-      <c r="E752" s="1"/>
-      <c r="F752" s="1"/>
-      <c r="G752" s="1"/>
-      <c r="H752" s="1"/>
+      <c r="B752" s="5"/>
+      <c r="C752" s="5"/>
+      <c r="D752" s="5"/>
+      <c r="E752" s="5"/>
+      <c r="F752" s="5"/>
+      <c r="G752" s="5"/>
+      <c r="H752" s="5"/>
     </row>
     <row r="753" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A753" t="s">
@@ -19109,6 +19109,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="I144:I147"/>
     <mergeCell ref="A172:H172"/>
     <mergeCell ref="A528:H528"/>
     <mergeCell ref="A585:H585"/>
@@ -19120,11 +19125,6 @@
     <mergeCell ref="A353:H353"/>
     <mergeCell ref="A411:H411"/>
     <mergeCell ref="A463:H463"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="I144:I147"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -19139,16 +19139,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -22489,16 +22489,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -24939,10 +24939,10 @@
       <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="J1" s="1"/>
+      <c r="J1" s="5"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -25215,10 +25215,10 @@
       <c r="G11">
         <v>42659.163342900007</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -26629,25 +26629,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="4" t="s">
+      <c r="A1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>7</v>
       </c>
       <c r="H1" t="s">
@@ -26661,27 +26661,27 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="B2" s="2">
-        <f>C2+E2</f>
+      <c r="B2" s="1">
+        <f t="shared" ref="B2:B14" si="0">C2+E2</f>
         <v>2</v>
       </c>
-      <c r="C2" s="2">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
         <v>18459.530451139999</v>
       </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3">
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2">
         <v>31614.260000000002</v>
       </c>
-      <c r="G2" s="3">
-        <f>D2+F2</f>
+      <c r="G2" s="2">
+        <f t="shared" ref="G2:G14" si="1">D2+F2</f>
         <v>50073.790451139997</v>
       </c>
       <c r="H2" t="s">
@@ -26696,27 +26696,27 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B3" s="2">
-        <f>C3+E3</f>
+      <c r="B3" s="1">
+        <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="C3" s="2">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3">
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
         <v>56188.060129739999</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>0.5</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <v>28021.74</v>
       </c>
-      <c r="G3" s="3">
-        <f>D3+F3</f>
+      <c r="G3" s="2">
+        <f t="shared" si="1"/>
         <v>84209.800129740004</v>
       </c>
       <c r="H3" t="s">
@@ -26731,27 +26731,27 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2">
-        <f>C4+E4</f>
+      <c r="B4" s="1">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="C4" s="2">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3">
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
         <v>43178.236515324999</v>
       </c>
-      <c r="E4" s="2">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3">
+      <c r="E4" s="1">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2">
         <v>26734.33</v>
       </c>
-      <c r="G4" s="3">
-        <f>D4+F4</f>
+      <c r="G4" s="2">
+        <f t="shared" si="1"/>
         <v>69912.566515325001</v>
       </c>
       <c r="H4" t="s">
@@ -26766,27 +26766,27 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B5" s="2">
-        <f>C5+E5</f>
+      <c r="B5" s="1">
+        <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="C5" s="1">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
         <v>0.5</v>
       </c>
-      <c r="F5" s="3">
+      <c r="F5" s="2">
         <v>23043.64</v>
       </c>
-      <c r="G5" s="3">
-        <f>D5+F5</f>
+      <c r="G5" s="2">
+        <f t="shared" si="1"/>
         <v>23043.64</v>
       </c>
       <c r="H5" t="s">
@@ -26801,27 +26801,27 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="2">
-        <f>C6+E6</f>
+      <c r="B6" s="1">
+        <f t="shared" si="0"/>
         <v>2.5</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>2</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="2">
         <v>107846.57343348001</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <v>0.5</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="2">
         <v>4650.3900000000003</v>
       </c>
-      <c r="G6" s="3">
-        <f>D6+F6</f>
+      <c r="G6" s="2">
+        <f t="shared" si="1"/>
         <v>112496.96343348001</v>
       </c>
       <c r="H6" t="s">
@@ -26836,27 +26836,27 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="2">
-        <f>C7+E7</f>
+      <c r="B7" s="1">
+        <f t="shared" si="0"/>
         <v>0.5</v>
       </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="C7" s="1">
+        <v>0</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
         <v>0.5</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F7" s="2">
         <v>1522.5999999999997</v>
       </c>
-      <c r="G7" s="3">
-        <f>D7+F7</f>
+      <c r="G7" s="2">
+        <f t="shared" si="1"/>
         <v>1522.5999999999997</v>
       </c>
       <c r="H7" t="s">
@@ -26871,27 +26871,27 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B8" s="2">
-        <f>C8+E8</f>
+      <c r="B8" s="1">
+        <f t="shared" si="0"/>
         <v>1.5</v>
       </c>
-      <c r="C8" s="2">
-        <v>1</v>
-      </c>
-      <c r="D8" s="3">
+      <c r="C8" s="1">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
         <v>1791.2760122400002</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <v>0.5</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="2">
         <v>739.46999999999991</v>
       </c>
-      <c r="G8" s="3">
-        <f>D8+F8</f>
+      <c r="G8" s="2">
+        <f t="shared" si="1"/>
         <v>2530.7460122400003</v>
       </c>
       <c r="H8" t="s">
@@ -26905,27 +26905,27 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="2">
-        <f>C9+E9</f>
-        <v>1</v>
-      </c>
-      <c r="C9" s="2">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="B9" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
         <v>73579.672848300004</v>
       </c>
-      <c r="E9" s="2">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3">
-        <v>0</v>
-      </c>
-      <c r="G9" s="3">
-        <f>D9+F9</f>
+      <c r="E9" s="1">
+        <v>0</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2">
+        <f t="shared" si="1"/>
         <v>73579.672848300004</v>
       </c>
       <c r="H9" t="s">
@@ -26939,27 +26939,27 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B10" s="2">
-        <f>C10+E10</f>
+      <c r="B10" s="1">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>3</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="2">
         <v>42694.97923692</v>
       </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-      <c r="F10" s="3">
-        <v>0</v>
-      </c>
-      <c r="G10" s="3">
-        <f>D10+F10</f>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="1"/>
         <v>42694.97923692</v>
       </c>
       <c r="H10" t="s">
@@ -26973,59 +26973,59 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="2">
-        <f>C11+E11</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="2">
-        <v>1</v>
-      </c>
-      <c r="D11" s="3">
+      <c r="B11" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
         <v>33164.673422275002</v>
       </c>
-      <c r="E11" s="2">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
-        <f>D11+F11</f>
+      <c r="E11" s="1">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2">
+        <f t="shared" si="1"/>
         <v>33164.673422275002</v>
       </c>
       <c r="H11" t="s">
         <v>258</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="B12" s="2">
-        <f>C12+E12</f>
+      <c r="B12" s="1">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>4</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="2">
         <v>29357.171238035</v>
       </c>
-      <c r="E12" s="2">
-        <v>0</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3">
-        <f>D12+F12</f>
+      <c r="E12" s="1">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2">
+        <f t="shared" si="1"/>
         <v>29357.171238035</v>
       </c>
       <c r="H12" t="s">
@@ -27039,27 +27039,27 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="2">
-        <f>C13+E13</f>
+      <c r="B13" s="1">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>2</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="2">
         <v>9690.1819726499998</v>
       </c>
-      <c r="E13" s="2">
-        <v>0</v>
-      </c>
-      <c r="F13" s="3">
-        <v>0</v>
-      </c>
-      <c r="G13" s="3">
-        <f>D13+F13</f>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" si="1"/>
         <v>9690.1819726499998</v>
       </c>
       <c r="H13" t="s">
@@ -27073,27 +27073,27 @@
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="2">
-        <f>C14+E14</f>
-        <v>1</v>
-      </c>
-      <c r="C14" s="2">
-        <v>1</v>
-      </c>
-      <c r="D14" s="3">
+      <c r="B14" s="1">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2">
         <v>1773.8949732200001</v>
       </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-      <c r="F14" s="3">
-        <v>0</v>
-      </c>
-      <c r="G14" s="3">
-        <f>D14+F14</f>
+      <c r="E14" s="1">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" si="1"/>
         <v>1773.8949732200001</v>
       </c>
       <c r="H14" t="s">

</xml_diff>

<commit_message>
fix: Corregir montos históricos Meta 24M (Abril - Julio)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
+++ b/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/VENTAS_MENSUALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3626C529-91B5-C149-9FDB-4DBFC633F59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83E12B-C311-1040-A6C0-8859FA8B95AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas Mensuales " sheetId="1" r:id="rId1"/>
@@ -19109,11 +19109,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="I144:I147"/>
     <mergeCell ref="A172:H172"/>
     <mergeCell ref="A528:H528"/>
     <mergeCell ref="A585:H585"/>
@@ -19125,6 +19120,11 @@
     <mergeCell ref="A353:H353"/>
     <mergeCell ref="A411:H411"/>
     <mergeCell ref="A463:H463"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="I144:I147"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-08-26 13:14)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
+++ b/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/VENTAS_MENSUALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83E12B-C311-1040-A6C0-8859FA8B95AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013312DF-4106-8946-8839-36590704856C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6140" yWindow="920" windowWidth="24480" windowHeight="16140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas Mensuales " sheetId="1" r:id="rId1"/>
@@ -926,13 +926,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -19109,6 +19110,11 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="I144:I147"/>
     <mergeCell ref="A172:H172"/>
     <mergeCell ref="A528:H528"/>
     <mergeCell ref="A585:H585"/>
@@ -19120,11 +19126,6 @@
     <mergeCell ref="A353:H353"/>
     <mergeCell ref="A411:H411"/>
     <mergeCell ref="A463:H463"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="I144:I147"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -26626,6 +26627,7 @@
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.1640625" customWidth="1"/>
+    <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -26690,7 +26692,7 @@
       <c r="I2" t="s">
         <v>244</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="6">
         <f>SUM(D2:D14)</f>
         <v>417724.25023332506</v>
       </c>
@@ -26760,7 +26762,7 @@
       <c r="I4" t="s">
         <v>246</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="6">
         <f>SUM(F2:F14)</f>
         <v>116326.43000000001</v>
       </c>
@@ -26865,7 +26867,7 @@
       <c r="I7" t="s">
         <v>249</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="6">
         <f>SUM(G2:G14)</f>
         <v>534050.68023332499</v>
       </c>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-02 12:54)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
+++ b/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/VENTAS_MENSUALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013312DF-4106-8946-8839-36590704856C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1689A6E-ACF9-4B46-91F9-B9330F7B2260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6140" yWindow="920" windowWidth="24480" windowHeight="16140" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ventas Mensuales " sheetId="1" r:id="rId1"/>
@@ -20,9 +20,12 @@
     <sheet name="JUNIO_CORREGIDO " sheetId="5" r:id="rId5"/>
     <sheet name="JULIO" sheetId="6" r:id="rId6"/>
     <sheet name="JULIO_CORREGIDO" sheetId="7" r:id="rId7"/>
+    <sheet name="AGOSTO" sheetId="8" r:id="rId8"/>
+    <sheet name="AGOSTO_CORREGIDO" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">JULIO_CORREGIDO!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">AGOSTO_CORREGIDO!$A$1:$G$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">JULIO_CORREGIDO!A1:G19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'JUNIO_CORREGIDO '!A1:G47</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">MAYO_CORREGIDO!A1:G47</definedName>
   </definedNames>
@@ -66,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2149" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2309" uniqueCount="271">
   <si>
     <t>Ventas mensuales Enero</t>
   </si>
@@ -859,6 +862,27 @@
   <si>
     <t>darinka</t>
   </si>
+  <si>
+    <t>OSCAR RAMIREZ RUIZ 119223</t>
+  </si>
+  <si>
+    <t>LUIS ANTONIO SALAZAR ESPINOSA 119447</t>
+  </si>
+  <si>
+    <t>PAULA ANGELICA LOMELI CAZARES 116876</t>
+  </si>
+  <si>
+    <t>LUIS ANTONIO SALAZAR ESPINOSA</t>
+  </si>
+  <si>
+    <t>OSCAR RAMIREZ RUIZ</t>
+  </si>
+  <si>
+    <t>PAU LOMELI</t>
+  </si>
+  <si>
+    <t>ANTEMIO</t>
+  </si>
 </sst>
 </file>
 
@@ -883,22 +907,28 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
-      <color theme="1"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -906,34 +936,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1273,16 +1285,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -2185,16 +2197,16 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-      <c r="E48" s="5"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -3124,16 +3136,16 @@
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="5" t="s">
+      <c r="A94" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B94" s="5"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="5"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-      <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
+      <c r="D94" s="1"/>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1"/>
+      <c r="G94" s="1"/>
+      <c r="H94" s="1"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
@@ -4068,16 +4080,16 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A134" s="5" t="s">
+      <c r="A134" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B134" s="5"/>
-      <c r="C134" s="5"/>
-      <c r="D134" s="5"/>
-      <c r="E134" s="5"/>
-      <c r="F134" s="5"/>
-      <c r="G134" s="5"/>
-      <c r="H134" s="5"/>
+      <c r="B134" s="1"/>
+      <c r="C134" s="1"/>
+      <c r="D134" s="1"/>
+      <c r="E134" s="1"/>
+      <c r="F134" s="1"/>
+      <c r="G134" s="1"/>
+      <c r="H134" s="1"/>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
@@ -4353,7 +4365,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I144" s="5" t="s">
+      <c r="I144" s="1" t="s">
         <v>69</v>
       </c>
       <c r="K144" t="s">
@@ -4378,7 +4390,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I145" s="5"/>
+      <c r="I145" s="1"/>
       <c r="K145" t="s">
         <v>66</v>
       </c>
@@ -4407,7 +4419,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I146" s="5"/>
+      <c r="I146" s="1"/>
       <c r="K146" t="s">
         <v>75</v>
       </c>
@@ -4436,7 +4448,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I147" s="5"/>
+      <c r="I147" s="1"/>
       <c r="K147" t="s">
         <v>79</v>
       </c>
@@ -4929,16 +4941,16 @@
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A172" s="5" t="s">
+      <c r="A172" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B172" s="5"/>
-      <c r="C172" s="5"/>
-      <c r="D172" s="5"/>
-      <c r="E172" s="5"/>
-      <c r="F172" s="5"/>
-      <c r="G172" s="5"/>
-      <c r="H172" s="5"/>
+      <c r="B172" s="1"/>
+      <c r="C172" s="1"/>
+      <c r="D172" s="1"/>
+      <c r="E172" s="1"/>
+      <c r="F172" s="1"/>
+      <c r="G172" s="1"/>
+      <c r="H172" s="1"/>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
@@ -5761,16 +5773,16 @@
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A212" s="5" t="s">
+      <c r="A212" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B212" s="5"/>
-      <c r="C212" s="5"/>
-      <c r="D212" s="5"/>
-      <c r="E212" s="5"/>
-      <c r="F212" s="5"/>
-      <c r="G212" s="5"/>
-      <c r="H212" s="5"/>
+      <c r="B212" s="1"/>
+      <c r="C212" s="1"/>
+      <c r="D212" s="1"/>
+      <c r="E212" s="1"/>
+      <c r="F212" s="1"/>
+      <c r="G212" s="1"/>
+      <c r="H212" s="1"/>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
@@ -6608,16 +6620,16 @@
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A254" s="5" t="s">
+      <c r="A254" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B254" s="5"/>
-      <c r="C254" s="5"/>
-      <c r="D254" s="5"/>
-      <c r="E254" s="5"/>
-      <c r="F254" s="5"/>
-      <c r="G254" s="5"/>
-      <c r="H254" s="5"/>
+      <c r="B254" s="1"/>
+      <c r="C254" s="1"/>
+      <c r="D254" s="1"/>
+      <c r="E254" s="1"/>
+      <c r="F254" s="1"/>
+      <c r="G254" s="1"/>
+      <c r="H254" s="1"/>
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
@@ -7543,16 +7555,16 @@
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A302" s="5" t="s">
+      <c r="A302" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B302" s="5"/>
-      <c r="C302" s="5"/>
-      <c r="D302" s="5"/>
-      <c r="E302" s="5"/>
-      <c r="F302" s="5"/>
-      <c r="G302" s="5"/>
-      <c r="H302" s="5"/>
+      <c r="B302" s="1"/>
+      <c r="C302" s="1"/>
+      <c r="D302" s="1"/>
+      <c r="E302" s="1"/>
+      <c r="F302" s="1"/>
+      <c r="G302" s="1"/>
+      <c r="H302" s="1"/>
     </row>
     <row r="303" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
@@ -8548,16 +8560,16 @@
       </c>
     </row>
     <row r="353" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A353" s="5" t="s">
+      <c r="A353" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="B353" s="5"/>
-      <c r="C353" s="5"/>
-      <c r="D353" s="5"/>
-      <c r="E353" s="5"/>
-      <c r="F353" s="5"/>
-      <c r="G353" s="5"/>
-      <c r="H353" s="5"/>
+      <c r="B353" s="1"/>
+      <c r="C353" s="1"/>
+      <c r="D353" s="1"/>
+      <c r="E353" s="1"/>
+      <c r="F353" s="1"/>
+      <c r="G353" s="1"/>
+      <c r="H353" s="1"/>
     </row>
     <row r="354" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
@@ -9616,16 +9628,16 @@
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A411" s="5" t="s">
+      <c r="A411" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B411" s="5"/>
-      <c r="C411" s="5"/>
-      <c r="D411" s="5"/>
-      <c r="E411" s="5"/>
-      <c r="F411" s="5"/>
-      <c r="G411" s="5"/>
-      <c r="H411" s="5"/>
+      <c r="B411" s="1"/>
+      <c r="C411" s="1"/>
+      <c r="D411" s="1"/>
+      <c r="E411" s="1"/>
+      <c r="F411" s="1"/>
+      <c r="G411" s="1"/>
+      <c r="H411" s="1"/>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
@@ -10719,16 +10731,16 @@
       </c>
     </row>
     <row r="463" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A463" s="5" t="s">
+      <c r="A463" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="B463" s="5"/>
-      <c r="C463" s="5"/>
-      <c r="D463" s="5"/>
-      <c r="E463" s="5"/>
-      <c r="F463" s="5"/>
-      <c r="G463" s="5"/>
-      <c r="H463" s="5"/>
+      <c r="B463" s="1"/>
+      <c r="C463" s="1"/>
+      <c r="D463" s="1"/>
+      <c r="E463" s="1"/>
+      <c r="F463" s="1"/>
+      <c r="G463" s="1"/>
+      <c r="H463" s="1"/>
     </row>
     <row r="464" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
@@ -12033,16 +12045,16 @@
       </c>
     </row>
     <row r="528" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A528" s="5" t="s">
+      <c r="A528" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="B528" s="5"/>
-      <c r="C528" s="5"/>
-      <c r="D528" s="5"/>
-      <c r="E528" s="5"/>
-      <c r="F528" s="5"/>
-      <c r="G528" s="5"/>
-      <c r="H528" s="5"/>
+      <c r="B528" s="1"/>
+      <c r="C528" s="1"/>
+      <c r="D528" s="1"/>
+      <c r="E528" s="1"/>
+      <c r="F528" s="1"/>
+      <c r="G528" s="1"/>
+      <c r="H528" s="1"/>
     </row>
     <row r="529" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A529" t="s">
@@ -13366,16 +13378,16 @@
       </c>
     </row>
     <row r="585" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A585" s="5" t="s">
+      <c r="A585" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B585" s="5"/>
-      <c r="C585" s="5"/>
-      <c r="D585" s="5"/>
-      <c r="E585" s="5"/>
-      <c r="F585" s="5"/>
-      <c r="G585" s="5"/>
-      <c r="H585" s="5"/>
+      <c r="B585" s="1"/>
+      <c r="C585" s="1"/>
+      <c r="D585" s="1"/>
+      <c r="E585" s="1"/>
+      <c r="F585" s="1"/>
+      <c r="G585" s="1"/>
+      <c r="H585" s="1"/>
     </row>
     <row r="586" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
@@ -15053,16 +15065,16 @@
       </c>
     </row>
     <row r="667" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A667" s="5" t="s">
+      <c r="A667" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B667" s="5"/>
-      <c r="C667" s="5"/>
-      <c r="D667" s="5"/>
-      <c r="E667" s="5"/>
-      <c r="F667" s="5"/>
-      <c r="G667" s="5"/>
-      <c r="H667" s="5"/>
+      <c r="B667" s="1"/>
+      <c r="C667" s="1"/>
+      <c r="D667" s="1"/>
+      <c r="E667" s="1"/>
+      <c r="F667" s="1"/>
+      <c r="G667" s="1"/>
+      <c r="H667" s="1"/>
     </row>
     <row r="668" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A668" t="s">
@@ -16798,16 +16810,16 @@
       </c>
     </row>
     <row r="752" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A752" s="5" t="s">
+      <c r="A752" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B752" s="5"/>
-      <c r="C752" s="5"/>
-      <c r="D752" s="5"/>
-      <c r="E752" s="5"/>
-      <c r="F752" s="5"/>
-      <c r="G752" s="5"/>
-      <c r="H752" s="5"/>
+      <c r="B752" s="1"/>
+      <c r="C752" s="1"/>
+      <c r="D752" s="1"/>
+      <c r="E752" s="1"/>
+      <c r="F752" s="1"/>
+      <c r="G752" s="1"/>
+      <c r="H752" s="1"/>
     </row>
     <row r="753" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A753" t="s">
@@ -19140,16 +19152,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -22490,16 +22502,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -24940,10 +24952,10 @@
       <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="J1" s="5"/>
+      <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -25216,10 +25228,10 @@
       <c r="G11">
         <v>42659.163342900007</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="5"/>
+      <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -26621,12 +26633,1071 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" t="s">
+        <v>258</v>
+      </c>
+      <c r="I1" t="s">
+        <v>125</v>
+      </c>
+      <c r="J1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B2">
+        <f t="shared" ref="B2:B14" si="0">C2+E2</f>
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>18459.530451139999</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>31614.260000000002</v>
+      </c>
+      <c r="G2">
+        <f t="shared" ref="G2:G14" si="1">D2+F2</f>
+        <v>50073.790451139997</v>
+      </c>
+      <c r="H2" t="s">
+        <v>258</v>
+      </c>
+      <c r="I2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J2">
+        <f>SUM(D2:D14)</f>
+        <v>417724.25023332506</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>56188.060129739999</v>
+      </c>
+      <c r="E3">
+        <v>0.5</v>
+      </c>
+      <c r="F3">
+        <v>28021.74</v>
+      </c>
+      <c r="G3">
+        <f t="shared" si="1"/>
+        <v>84209.800129740004</v>
+      </c>
+      <c r="H3" t="s">
+        <v>258</v>
+      </c>
+      <c r="I3" t="s">
+        <v>245</v>
+      </c>
+      <c r="J3">
+        <f>SUM(C2:C14)</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>43178.236515324999</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>26734.33</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="1"/>
+        <v>69912.566515325001</v>
+      </c>
+      <c r="H4" t="s">
+        <v>258</v>
+      </c>
+      <c r="I4" t="s">
+        <v>246</v>
+      </c>
+      <c r="J4">
+        <f>SUM(F2:F14)</f>
+        <v>116326.43000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>210</v>
+      </c>
+      <c r="B5">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0.5</v>
+      </c>
+      <c r="F5">
+        <v>23043.64</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="1"/>
+        <v>23043.64</v>
+      </c>
+      <c r="H5" t="s">
+        <v>258</v>
+      </c>
+      <c r="I5" t="s">
+        <v>247</v>
+      </c>
+      <c r="J5">
+        <f>SUM(E2:E14)</f>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>107846.57343348001</v>
+      </c>
+      <c r="E6">
+        <v>0.5</v>
+      </c>
+      <c r="F6">
+        <v>4650.3900000000003</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="1"/>
+        <v>112496.96343348001</v>
+      </c>
+      <c r="H6" t="s">
+        <v>258</v>
+      </c>
+      <c r="I6" t="s">
+        <v>248</v>
+      </c>
+      <c r="J6">
+        <f>SUM(B2:B14)</f>
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0.5</v>
+      </c>
+      <c r="F7">
+        <v>1522.5999999999997</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="1"/>
+        <v>1522.5999999999997</v>
+      </c>
+      <c r="H7" t="s">
+        <v>258</v>
+      </c>
+      <c r="I7" t="s">
+        <v>249</v>
+      </c>
+      <c r="J7">
+        <f>SUM(G2:G14)</f>
+        <v>534050.68023332499</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>1791.2760122400002</v>
+      </c>
+      <c r="E8">
+        <v>0.5</v>
+      </c>
+      <c r="F8">
+        <v>739.46999999999991</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="1"/>
+        <v>2530.7460122400003</v>
+      </c>
+      <c r="H8" t="s">
+        <v>258</v>
+      </c>
+      <c r="I8" t="s">
+        <v>258</v>
+      </c>
+      <c r="J8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>73579.672848300004</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="1"/>
+        <v>73579.672848300004</v>
+      </c>
+      <c r="H9" t="s">
+        <v>258</v>
+      </c>
+      <c r="I9" t="s">
+        <v>258</v>
+      </c>
+      <c r="J9" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>42694.97923692</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="1"/>
+        <v>42694.97923692</v>
+      </c>
+      <c r="H10" t="s">
+        <v>258</v>
+      </c>
+      <c r="I10" t="s">
+        <v>258</v>
+      </c>
+      <c r="J10" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>33164.673422275002</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="1"/>
+        <v>33164.673422275002</v>
+      </c>
+      <c r="H11" t="s">
+        <v>258</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>225</v>
+      </c>
+      <c r="B12">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12">
+        <v>29357.171238035</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="1"/>
+        <v>29357.171238035</v>
+      </c>
+      <c r="H12" t="s">
+        <v>258</v>
+      </c>
+      <c r="I12" t="s">
+        <v>132</v>
+      </c>
+      <c r="J12" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>130</v>
+      </c>
+      <c r="B13">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>9690.1819726499998</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="1"/>
+        <v>9690.1819726499998</v>
+      </c>
+      <c r="H13" t="s">
+        <v>258</v>
+      </c>
+      <c r="I13" t="s">
+        <v>134</v>
+      </c>
+      <c r="J13" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
+        <v>1773.8949732200001</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="1"/>
+        <v>1773.8949732200001</v>
+      </c>
+      <c r="H14" t="s">
+        <v>258</v>
+      </c>
+      <c r="I14" t="s">
+        <v>136</v>
+      </c>
+      <c r="J14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I15" t="s">
+        <v>137</v>
+      </c>
+      <c r="J15" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="I16" t="s">
+        <v>138</v>
+      </c>
+      <c r="J16" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="I17" t="s">
+        <v>140</v>
+      </c>
+      <c r="J17" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="18" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="I18" t="s">
+        <v>141</v>
+      </c>
+      <c r="J18" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="19" spans="9:10" x14ac:dyDescent="0.2">
+      <c r="I19" t="s">
+        <v>143</v>
+      </c>
+      <c r="J19" t="s">
+        <v>263</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G19" xr:uid="{00000000-0009-0000-0000-000006000000}"/>
+  <mergeCells count="1">
+    <mergeCell ref="I11:J11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:J19" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="4" max="5" width="11.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>187</v>
+      </c>
+      <c r="B1" t="s">
+        <v>188</v>
+      </c>
+      <c r="C1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H1" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="2">
+        <v>28355.0347050036</v>
+      </c>
+      <c r="E2" s="2">
+        <f t="shared" ref="E2:E26" si="0">D2/IF(B2="MENSUAL",12,IF(B2="TRIMESTRAL",4,IF(B2="SEMESTRAL",2,1)))</f>
+        <v>2362.9195587503</v>
+      </c>
+      <c r="G2" t="s">
+        <v>244</v>
+      </c>
+      <c r="H2">
+        <f>SUMIF(C2:C26,"VIDA",E2:E26)</f>
+        <v>563907.97513739287</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" t="s">
+        <v>197</v>
+      </c>
+      <c r="D3" s="2">
+        <v>24718.650359059997</v>
+      </c>
+      <c r="E3" s="2">
+        <f t="shared" si="0"/>
+        <v>12359.325179529998</v>
+      </c>
+      <c r="G3" t="s">
+        <v>246</v>
+      </c>
+      <c r="H3">
+        <f>SUMIF(C2:C26,"GMM",E2:E26)</f>
+        <v>37128.26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B4" t="s">
+        <v>198</v>
+      </c>
+      <c r="C4" t="s">
+        <v>197</v>
+      </c>
+      <c r="D4" s="2">
+        <v>96899.18338314</v>
+      </c>
+      <c r="E4" s="2">
+        <f t="shared" si="0"/>
+        <v>96899.18338314</v>
+      </c>
+      <c r="G4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H4">
+        <f>COUNTIF(C2:C26,"GMM")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>195</v>
+      </c>
+      <c r="B5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" t="s">
+        <v>197</v>
+      </c>
+      <c r="D5" s="2">
+        <v>66100.985070369992</v>
+      </c>
+      <c r="E5" s="2">
+        <f t="shared" si="0"/>
+        <v>66100.985070369992</v>
+      </c>
+      <c r="G5" t="s">
+        <v>245</v>
+      </c>
+      <c r="H5">
+        <f>COUNTIF(C2:C26,"VIDA")</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D6" s="2">
+        <v>33322.854766909993</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" si="0"/>
+        <v>33322.854766909993</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7" t="s">
+        <v>199</v>
+      </c>
+      <c r="C7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" s="2">
+        <v>73112.783475479999</v>
+      </c>
+      <c r="E7" s="2">
+        <f t="shared" si="0"/>
+        <v>6092.7319562900002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>229</v>
+      </c>
+      <c r="B8" t="s">
+        <v>199</v>
+      </c>
+      <c r="C8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="2">
+        <v>23580.417253862401</v>
+      </c>
+      <c r="E8" s="2">
+        <f t="shared" si="0"/>
+        <v>1965.0347711552001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>229</v>
+      </c>
+      <c r="B9" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" t="s">
+        <v>194</v>
+      </c>
+      <c r="D9" s="2">
+        <v>65420.399999999994</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="0"/>
+        <v>5451.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>243</v>
+      </c>
+      <c r="B10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C10" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" s="2">
+        <v>90033.454256679994</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>90033.454256679994</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" t="s">
+        <v>199</v>
+      </c>
+      <c r="C11" t="s">
+        <v>197</v>
+      </c>
+      <c r="D11" s="2">
+        <v>23527.39078944</v>
+      </c>
+      <c r="E11" s="2">
+        <f t="shared" si="0"/>
+        <v>1960.61589912</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C12" t="s">
+        <v>194</v>
+      </c>
+      <c r="D12" s="2">
+        <v>27662.28</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="0"/>
+        <v>2305.19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B13" t="s">
+        <v>198</v>
+      </c>
+      <c r="C13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D13" s="2">
+        <v>83019.199999999997</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="0"/>
+        <v>83019.199999999997</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C14" t="s">
+        <v>197</v>
+      </c>
+      <c r="D14" s="2">
+        <v>36338.399738128799</v>
+      </c>
+      <c r="E14" s="2">
+        <f t="shared" si="0"/>
+        <v>3028.1999781773998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B15" t="s">
+        <v>198</v>
+      </c>
+      <c r="C15" t="s">
+        <v>197</v>
+      </c>
+      <c r="D15" s="2">
+        <v>58335.862101919993</v>
+      </c>
+      <c r="E15" s="2">
+        <f t="shared" si="0"/>
+        <v>58335.862101919993</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>264</v>
+      </c>
+      <c r="B16" t="s">
+        <v>199</v>
+      </c>
+      <c r="C16" t="s">
+        <v>197</v>
+      </c>
+      <c r="D16" s="2">
+        <v>28766.235240000005</v>
+      </c>
+      <c r="E16" s="2">
+        <f t="shared" si="0"/>
+        <v>2397.1862700000006</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>167</v>
+      </c>
+      <c r="B17" t="s">
+        <v>198</v>
+      </c>
+      <c r="C17" t="s">
+        <v>197</v>
+      </c>
+      <c r="D17" s="2">
+        <v>34327.825434270002</v>
+      </c>
+      <c r="E17" s="2">
+        <f t="shared" si="0"/>
+        <v>34327.825434270002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" t="s">
+        <v>198</v>
+      </c>
+      <c r="C18" t="s">
+        <v>197</v>
+      </c>
+      <c r="D18" s="2">
+        <v>29809.2060079</v>
+      </c>
+      <c r="E18" s="2">
+        <f t="shared" si="0"/>
+        <v>29809.2060079</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>167</v>
+      </c>
+      <c r="B19" t="s">
+        <v>198</v>
+      </c>
+      <c r="C19" t="s">
+        <v>194</v>
+      </c>
+      <c r="D19" s="2">
+        <v>26627.46</v>
+      </c>
+      <c r="E19" s="2">
+        <f t="shared" si="0"/>
+        <v>26627.46</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>265</v>
+      </c>
+      <c r="B20" t="s">
+        <v>199</v>
+      </c>
+      <c r="C20" t="s">
+        <v>197</v>
+      </c>
+      <c r="D20" s="2">
+        <v>36672.004980719998</v>
+      </c>
+      <c r="E20" s="2">
+        <f t="shared" si="0"/>
+        <v>3056.0004150599998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>265</v>
+      </c>
+      <c r="B21" t="s">
+        <v>199</v>
+      </c>
+      <c r="C21" t="s">
+        <v>197</v>
+      </c>
+      <c r="D21" s="2">
+        <v>20910.710278080001</v>
+      </c>
+      <c r="E21" s="2">
+        <f t="shared" si="0"/>
+        <v>1742.55918984</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>259</v>
+      </c>
+      <c r="B22" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" t="s">
+        <v>197</v>
+      </c>
+      <c r="D22" s="2">
+        <v>36755.186497499999</v>
+      </c>
+      <c r="E22" s="2">
+        <f t="shared" si="0"/>
+        <v>18377.593248749999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>259</v>
+      </c>
+      <c r="B23" t="s">
+        <v>199</v>
+      </c>
+      <c r="C23" t="s">
+        <v>194</v>
+      </c>
+      <c r="D23" s="2">
+        <v>24314.639999999999</v>
+      </c>
+      <c r="E23" s="2">
+        <f t="shared" si="0"/>
+        <v>2026.22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>266</v>
+      </c>
+      <c r="B24" t="s">
+        <v>193</v>
+      </c>
+      <c r="C24" t="s">
+        <v>197</v>
+      </c>
+      <c r="D24" s="2">
+        <v>32809.260598559995</v>
+      </c>
+      <c r="E24" s="2">
+        <f t="shared" si="0"/>
+        <v>16404.630299279997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>266</v>
+      </c>
+      <c r="B25" t="s">
+        <v>199</v>
+      </c>
+      <c r="C25" t="s">
+        <v>197</v>
+      </c>
+      <c r="D25" s="2">
+        <v>27751.288203000007</v>
+      </c>
+      <c r="E25" s="2">
+        <f t="shared" si="0"/>
+        <v>2312.6073502500008</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>261</v>
+      </c>
+      <c r="B26" t="s">
+        <v>199</v>
+      </c>
+      <c r="C26" t="s">
+        <v>194</v>
+      </c>
+      <c r="D26" s="2">
+        <v>8612.2800000000007</v>
+      </c>
+      <c r="E26" s="2">
+        <f t="shared" si="0"/>
+        <v>717.69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:H26" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="37.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.1640625" customWidth="1"/>
+    <col min="9" max="9" width="19.83203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -26640,22 +27711,22 @@
       <c r="C1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>122</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="H1" t="s">
         <v>258</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>125</v>
       </c>
       <c r="J1" t="s">
@@ -26663,238 +27734,218 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="1">
-        <f t="shared" ref="B2:B14" si="0">C2+E2</f>
+      <c r="A2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2">
         <v>2</v>
       </c>
-      <c r="C2" s="1">
-        <v>1</v>
+      <c r="C2">
+        <v>2</v>
       </c>
       <c r="D2" s="2">
-        <v>18459.530451139999</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1</v>
+        <v>163000.16845350998</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
       </c>
       <c r="F2" s="2">
-        <v>31614.260000000002</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2">
-        <f t="shared" ref="G2:G14" si="1">D2+F2</f>
-        <v>50073.790451139997</v>
+        <v>163000.16845350998</v>
       </c>
       <c r="H2" t="s">
         <v>258</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="J2" s="6">
-        <f>SUM(D2:D14)</f>
-        <v>417724.25023332506</v>
+      <c r="J2" s="2">
+        <v>563907.97513739299</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="B3" s="1">
-        <f t="shared" si="0"/>
-        <v>1.5</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1</v>
+      <c r="A3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B3">
+        <v>2.5</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
       </c>
       <c r="D3" s="2">
-        <v>56188.060129739999</v>
-      </c>
-      <c r="E3" s="1">
+        <v>64137.031442170002</v>
+      </c>
+      <c r="E3">
         <v>0.5</v>
       </c>
       <c r="F3" s="2">
-        <v>28021.74</v>
+        <v>26627.46</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" si="1"/>
-        <v>84209.800129740004</v>
+        <v>90764.491442169994</v>
       </c>
       <c r="H3" t="s">
         <v>258</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="3" t="s">
         <v>245</v>
       </c>
       <c r="J3">
-        <f>SUM(C2:C14)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="1">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" s="2">
-        <v>43178.236515324999</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1</v>
+        <v>90033.454256679994</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
       </c>
       <c r="F4" s="2">
-        <v>26734.33</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2">
-        <f t="shared" si="1"/>
-        <v>69912.566515325001</v>
+        <v>90033.454256679994</v>
       </c>
       <c r="H4" t="s">
         <v>258</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="J4" s="6">
-        <f>SUM(F2:F14)</f>
-        <v>116326.43000000001</v>
+      <c r="J4" s="2">
+        <v>37128.26</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B5" s="1">
-        <f t="shared" si="0"/>
+      <c r="A5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5">
+        <v>2.5</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2">
+        <v>86047.399978177404</v>
+      </c>
+      <c r="E5">
         <v>0.5</v>
       </c>
-      <c r="C5" s="1">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0.5</v>
-      </c>
       <c r="F5" s="2">
-        <v>23043.64</v>
+        <v>2305.19</v>
       </c>
       <c r="G5" s="2">
-        <f t="shared" si="1"/>
-        <v>23043.64</v>
+        <v>88352.589978177406</v>
       </c>
       <c r="H5" t="s">
         <v>258</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="3" t="s">
         <v>247</v>
       </c>
       <c r="J5">
-        <f>SUM(E2:E14)</f>
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="1">
-        <f t="shared" si="0"/>
-        <v>2.5</v>
-      </c>
-      <c r="C6" s="1">
-        <v>2</v>
+      <c r="A6" t="s">
+        <v>186</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
       </c>
       <c r="D6" s="2">
-        <v>107846.57343348001</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0.5</v>
+        <v>58335.862101919993</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
       </c>
       <c r="F6" s="2">
-        <v>4650.3900000000003</v>
+        <v>0</v>
       </c>
       <c r="G6" s="2">
-        <f t="shared" si="1"/>
-        <v>112496.96343348001</v>
+        <v>58335.862101919993</v>
       </c>
       <c r="H6" t="s">
         <v>258</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="3" t="s">
         <v>248</v>
       </c>
       <c r="J6">
-        <f>SUM(B2:B14)</f>
         <v>22.5</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" s="1">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0</v>
+      <c r="A7" t="s">
+        <v>239</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
       </c>
       <c r="D7" s="2">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.5</v>
+        <v>33322.854766909993</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
       </c>
       <c r="F7" s="2">
-        <v>1522.5999999999997</v>
+        <v>0</v>
       </c>
       <c r="G7" s="2">
-        <f t="shared" si="1"/>
-        <v>1522.5999999999997</v>
+        <v>33322.854766909993</v>
       </c>
       <c r="H7" t="s">
         <v>258</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="J7" s="6">
-        <f>SUM(G2:G14)</f>
-        <v>534050.68023332499</v>
+      <c r="J7" s="2">
+        <v>601036.23513739277</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B8" s="1">
-        <f t="shared" si="0"/>
+      <c r="A8" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8">
         <v>1.5</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" s="2">
-        <v>1791.2760122400002</v>
-      </c>
-      <c r="E8" s="1">
+        <v>18377.593248749999</v>
+      </c>
+      <c r="E8">
         <v>0.5</v>
       </c>
       <c r="F8" s="2">
-        <v>739.46999999999991</v>
+        <v>2026.22</v>
       </c>
       <c r="G8" s="2">
-        <f t="shared" si="1"/>
-        <v>2530.7460122400003</v>
+        <v>20403.813248750001</v>
       </c>
       <c r="H8" t="s">
         <v>258</v>
@@ -26907,28 +27958,26 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="1">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="C9" s="1">
-        <v>1</v>
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
       </c>
       <c r="D9" s="2">
-        <v>73579.672848300004</v>
-      </c>
-      <c r="E9" s="1">
+        <v>18717.237649529998</v>
+      </c>
+      <c r="E9">
         <v>0</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
       </c>
       <c r="G9" s="2">
-        <f t="shared" si="1"/>
-        <v>73579.672848300004</v>
+        <v>18717.237649529998</v>
       </c>
       <c r="H9" t="s">
         <v>258</v>
@@ -26941,28 +27990,26 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B10" s="1">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="C10" s="1">
-        <v>3</v>
+      <c r="A10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
       </c>
       <c r="D10" s="2">
-        <v>42694.97923692</v>
-      </c>
-      <c r="E10" s="1">
+        <v>14722.244738280298</v>
+      </c>
+      <c r="E10">
         <v>0</v>
       </c>
       <c r="F10" s="2">
         <v>0</v>
       </c>
       <c r="G10" s="2">
-        <f t="shared" si="1"/>
-        <v>42694.97923692</v>
+        <v>14722.244738280298</v>
       </c>
       <c r="H10" t="s">
         <v>258</v>
@@ -26975,191 +28022,244 @@
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="1">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="C11" s="1">
+      <c r="A11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B11">
+        <v>1.5</v>
+      </c>
+      <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" s="2">
-        <v>33164.673422275002</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0</v>
+        <v>1965.0347711552001</v>
+      </c>
+      <c r="E11">
+        <v>0.5</v>
       </c>
       <c r="F11" s="2">
-        <v>0</v>
+        <v>5451.7</v>
       </c>
       <c r="G11" s="2">
-        <f t="shared" si="1"/>
-        <v>33164.673422275002</v>
+        <v>7416.7347711552002</v>
       </c>
       <c r="H11" t="s">
         <v>258</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="5"/>
+      <c r="J11" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="B12" s="1">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="C12" s="1">
-        <v>4</v>
+      <c r="A12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
       </c>
       <c r="D12" s="2">
-        <v>29357.171238035</v>
-      </c>
-      <c r="E12" s="1">
+        <v>6092.7319562900002</v>
+      </c>
+      <c r="E12">
         <v>0</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
       </c>
       <c r="G12" s="2">
-        <f t="shared" si="1"/>
-        <v>29357.171238035</v>
+        <v>6092.7319562900002</v>
       </c>
       <c r="H12" t="s">
         <v>258</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="3" t="s">
         <v>132</v>
       </c>
       <c r="J12" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="B13" s="1">
-        <f t="shared" si="0"/>
+      <c r="A13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B13">
         <v>2</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13">
         <v>2</v>
       </c>
       <c r="D13" s="2">
-        <v>9690.1819726499998</v>
-      </c>
-      <c r="E13" s="1">
+        <v>4798.5596048999996</v>
+      </c>
+      <c r="E13">
         <v>0</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
       </c>
       <c r="G13" s="2">
-        <f t="shared" si="1"/>
-        <v>9690.1819726499998</v>
+        <v>4798.5596048999996</v>
       </c>
       <c r="H13" t="s">
         <v>258</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="3" t="s">
         <v>134</v>
       </c>
       <c r="J13" t="s">
-        <v>238</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="1">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="C14" s="1">
+      <c r="A14" t="s">
+        <v>268</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" s="2">
-        <v>1773.8949732200001</v>
-      </c>
-      <c r="E14" s="1">
+        <v>2397.1862700000006</v>
+      </c>
+      <c r="E14">
         <v>0</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
       </c>
       <c r="G14" s="2">
-        <f t="shared" si="1"/>
-        <v>1773.8949732200001</v>
+        <v>2397.1862700000006</v>
       </c>
       <c r="H14" t="s">
         <v>258</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="3" t="s">
         <v>136</v>
       </c>
       <c r="J14" t="s">
-        <v>237</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I15" t="s">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2">
+        <v>1960.61589912</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1960.61589912</v>
+      </c>
+      <c r="H15" t="s">
+        <v>258</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>137</v>
       </c>
       <c r="J15" t="s">
-        <v>238</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="I16" t="s">
+      <c r="A16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B16">
+        <v>0.5</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0.5</v>
+      </c>
+      <c r="F16" s="2">
+        <v>717.69</v>
+      </c>
+      <c r="G16" s="2">
+        <v>717.69</v>
+      </c>
+      <c r="H16" t="s">
+        <v>258</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>138</v>
       </c>
       <c r="J16" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="17" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I17" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="17" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H17" t="s">
+        <v>258</v>
+      </c>
+      <c r="I17" s="3" t="s">
         <v>140</v>
       </c>
       <c r="J17" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="18" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H18" t="s">
+        <v>258</v>
+      </c>
+      <c r="I18" s="3" t="s">
         <v>141</v>
       </c>
       <c r="J18" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="19" spans="9:10" x14ac:dyDescent="0.2">
-      <c r="I19" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="19" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H19" t="s">
+        <v>258</v>
+      </c>
+      <c r="I19" s="3" t="s">
         <v>143</v>
       </c>
       <c r="J19" t="s">
-        <v>263</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0800-000000000000}">
+    <filterColumn colId="2">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G19">
-      <sortCondition descending="1" ref="F1:F19"/>
+      <sortCondition descending="1" ref="G1:G19"/>
     </sortState>
   </autoFilter>
-  <mergeCells count="1">
-    <mergeCell ref="I11:J11"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J1 H11:H14 H2:J10" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 H3:J11 H2:I2 H19:I19 H12:I12 H13:I13 H14:I14 H15:I15 H16:I16 H17:I17 H18:I18" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-09-03 14:29)
</commit_message>
<xml_diff>
--- a/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
+++ b/VENTAS_MENSUALES/VENTAS MENSUALES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/VENTAS_MENSUALES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1689A6E-ACF9-4B46-91F9-B9330F7B2260}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BE02EBC-2979-3148-9948-9169BC3AA187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="600" windowWidth="24480" windowHeight="16140" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2309" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2306" uniqueCount="270">
   <si>
     <t>Ventas mensuales Enero</t>
   </si>
@@ -878,9 +878,6 @@
     <t>OSCAR RAMIREZ RUIZ</t>
   </si>
   <si>
-    <t>PAU LOMELI</t>
-  </si>
-  <si>
     <t>ANTEMIO</t>
   </si>
 </sst>
@@ -943,9 +940,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1285,16 +1282,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -2197,16 +2194,16 @@
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+      <c r="A48" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -3136,16 +3133,16 @@
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A94" s="1" t="s">
+      <c r="A94" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B94" s="1"/>
-      <c r="C94" s="1"/>
-      <c r="D94" s="1"/>
-      <c r="E94" s="1"/>
-      <c r="F94" s="1"/>
-      <c r="G94" s="1"/>
-      <c r="H94" s="1"/>
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="H94" s="3"/>
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
@@ -4080,16 +4077,16 @@
       </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A134" s="1" t="s">
+      <c r="A134" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B134" s="1"/>
-      <c r="C134" s="1"/>
-      <c r="D134" s="1"/>
-      <c r="E134" s="1"/>
-      <c r="F134" s="1"/>
-      <c r="G134" s="1"/>
-      <c r="H134" s="1"/>
+      <c r="B134" s="3"/>
+      <c r="C134" s="3"/>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3"/>
+      <c r="G134" s="3"/>
+      <c r="H134" s="3"/>
     </row>
     <row r="135" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
@@ -4365,7 +4362,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I144" s="1" t="s">
+      <c r="I144" s="3" t="s">
         <v>69</v>
       </c>
       <c r="K144" t="s">
@@ -4390,7 +4387,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I145" s="1"/>
+      <c r="I145" s="3"/>
       <c r="K145" t="s">
         <v>66</v>
       </c>
@@ -4419,7 +4416,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I146" s="1"/>
+      <c r="I146" s="3"/>
       <c r="K146" t="s">
         <v>75</v>
       </c>
@@ -4448,7 +4445,7 @@
         <f>SUM(#REF!,#REF!)</f>
         <v>#REF!</v>
       </c>
-      <c r="I147" s="1"/>
+      <c r="I147" s="3"/>
       <c r="K147" t="s">
         <v>79</v>
       </c>
@@ -4941,16 +4938,16 @@
       </c>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A172" s="1" t="s">
+      <c r="A172" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B172" s="1"/>
-      <c r="C172" s="1"/>
-      <c r="D172" s="1"/>
-      <c r="E172" s="1"/>
-      <c r="F172" s="1"/>
-      <c r="G172" s="1"/>
-      <c r="H172" s="1"/>
+      <c r="B172" s="3"/>
+      <c r="C172" s="3"/>
+      <c r="D172" s="3"/>
+      <c r="E172" s="3"/>
+      <c r="F172" s="3"/>
+      <c r="G172" s="3"/>
+      <c r="H172" s="3"/>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
@@ -5773,16 +5770,16 @@
       </c>
     </row>
     <row r="212" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A212" s="1" t="s">
+      <c r="A212" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B212" s="1"/>
-      <c r="C212" s="1"/>
-      <c r="D212" s="1"/>
-      <c r="E212" s="1"/>
-      <c r="F212" s="1"/>
-      <c r="G212" s="1"/>
-      <c r="H212" s="1"/>
+      <c r="B212" s="3"/>
+      <c r="C212" s="3"/>
+      <c r="D212" s="3"/>
+      <c r="E212" s="3"/>
+      <c r="F212" s="3"/>
+      <c r="G212" s="3"/>
+      <c r="H212" s="3"/>
     </row>
     <row r="213" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
@@ -6620,16 +6617,16 @@
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A254" s="1" t="s">
+      <c r="A254" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B254" s="1"/>
-      <c r="C254" s="1"/>
-      <c r="D254" s="1"/>
-      <c r="E254" s="1"/>
-      <c r="F254" s="1"/>
-      <c r="G254" s="1"/>
-      <c r="H254" s="1"/>
+      <c r="B254" s="3"/>
+      <c r="C254" s="3"/>
+      <c r="D254" s="3"/>
+      <c r="E254" s="3"/>
+      <c r="F254" s="3"/>
+      <c r="G254" s="3"/>
+      <c r="H254" s="3"/>
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
@@ -7555,16 +7552,16 @@
       </c>
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A302" s="1" t="s">
+      <c r="A302" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B302" s="1"/>
-      <c r="C302" s="1"/>
-      <c r="D302" s="1"/>
-      <c r="E302" s="1"/>
-      <c r="F302" s="1"/>
-      <c r="G302" s="1"/>
-      <c r="H302" s="1"/>
+      <c r="B302" s="3"/>
+      <c r="C302" s="3"/>
+      <c r="D302" s="3"/>
+      <c r="E302" s="3"/>
+      <c r="F302" s="3"/>
+      <c r="G302" s="3"/>
+      <c r="H302" s="3"/>
     </row>
     <row r="303" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
@@ -8560,16 +8557,16 @@
       </c>
     </row>
     <row r="353" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A353" s="1" t="s">
+      <c r="A353" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B353" s="1"/>
-      <c r="C353" s="1"/>
-      <c r="D353" s="1"/>
-      <c r="E353" s="1"/>
-      <c r="F353" s="1"/>
-      <c r="G353" s="1"/>
-      <c r="H353" s="1"/>
+      <c r="B353" s="3"/>
+      <c r="C353" s="3"/>
+      <c r="D353" s="3"/>
+      <c r="E353" s="3"/>
+      <c r="F353" s="3"/>
+      <c r="G353" s="3"/>
+      <c r="H353" s="3"/>
     </row>
     <row r="354" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
@@ -9628,16 +9625,16 @@
       </c>
     </row>
     <row r="411" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A411" s="1" t="s">
+      <c r="A411" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B411" s="1"/>
-      <c r="C411" s="1"/>
-      <c r="D411" s="1"/>
-      <c r="E411" s="1"/>
-      <c r="F411" s="1"/>
-      <c r="G411" s="1"/>
-      <c r="H411" s="1"/>
+      <c r="B411" s="3"/>
+      <c r="C411" s="3"/>
+      <c r="D411" s="3"/>
+      <c r="E411" s="3"/>
+      <c r="F411" s="3"/>
+      <c r="G411" s="3"/>
+      <c r="H411" s="3"/>
     </row>
     <row r="412" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A412" t="s">
@@ -10731,16 +10728,16 @@
       </c>
     </row>
     <row r="463" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A463" s="1" t="s">
+      <c r="A463" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="B463" s="1"/>
-      <c r="C463" s="1"/>
-      <c r="D463" s="1"/>
-      <c r="E463" s="1"/>
-      <c r="F463" s="1"/>
-      <c r="G463" s="1"/>
-      <c r="H463" s="1"/>
+      <c r="B463" s="3"/>
+      <c r="C463" s="3"/>
+      <c r="D463" s="3"/>
+      <c r="E463" s="3"/>
+      <c r="F463" s="3"/>
+      <c r="G463" s="3"/>
+      <c r="H463" s="3"/>
     </row>
     <row r="464" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A464" t="s">
@@ -12045,16 +12042,16 @@
       </c>
     </row>
     <row r="528" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A528" s="1" t="s">
+      <c r="A528" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B528" s="1"/>
-      <c r="C528" s="1"/>
-      <c r="D528" s="1"/>
-      <c r="E528" s="1"/>
-      <c r="F528" s="1"/>
-      <c r="G528" s="1"/>
-      <c r="H528" s="1"/>
+      <c r="B528" s="3"/>
+      <c r="C528" s="3"/>
+      <c r="D528" s="3"/>
+      <c r="E528" s="3"/>
+      <c r="F528" s="3"/>
+      <c r="G528" s="3"/>
+      <c r="H528" s="3"/>
     </row>
     <row r="529" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A529" t="s">
@@ -13378,16 +13375,16 @@
       </c>
     </row>
     <row r="585" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A585" s="1" t="s">
+      <c r="A585" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B585" s="1"/>
-      <c r="C585" s="1"/>
-      <c r="D585" s="1"/>
-      <c r="E585" s="1"/>
-      <c r="F585" s="1"/>
-      <c r="G585" s="1"/>
-      <c r="H585" s="1"/>
+      <c r="B585" s="3"/>
+      <c r="C585" s="3"/>
+      <c r="D585" s="3"/>
+      <c r="E585" s="3"/>
+      <c r="F585" s="3"/>
+      <c r="G585" s="3"/>
+      <c r="H585" s="3"/>
     </row>
     <row r="586" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A586" t="s">
@@ -15065,16 +15062,16 @@
       </c>
     </row>
     <row r="667" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A667" s="1" t="s">
+      <c r="A667" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B667" s="1"/>
-      <c r="C667" s="1"/>
-      <c r="D667" s="1"/>
-      <c r="E667" s="1"/>
-      <c r="F667" s="1"/>
-      <c r="G667" s="1"/>
-      <c r="H667" s="1"/>
+      <c r="B667" s="3"/>
+      <c r="C667" s="3"/>
+      <c r="D667" s="3"/>
+      <c r="E667" s="3"/>
+      <c r="F667" s="3"/>
+      <c r="G667" s="3"/>
+      <c r="H667" s="3"/>
     </row>
     <row r="668" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A668" t="s">
@@ -16810,16 +16807,16 @@
       </c>
     </row>
     <row r="752" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A752" s="1" t="s">
+      <c r="A752" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B752" s="1"/>
-      <c r="C752" s="1"/>
-      <c r="D752" s="1"/>
-      <c r="E752" s="1"/>
-      <c r="F752" s="1"/>
-      <c r="G752" s="1"/>
-      <c r="H752" s="1"/>
+      <c r="B752" s="3"/>
+      <c r="C752" s="3"/>
+      <c r="D752" s="3"/>
+      <c r="E752" s="3"/>
+      <c r="F752" s="3"/>
+      <c r="G752" s="3"/>
+      <c r="H752" s="3"/>
     </row>
     <row r="753" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A753" t="s">
@@ -19122,11 +19119,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A94:H94"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="I144:I147"/>
     <mergeCell ref="A172:H172"/>
     <mergeCell ref="A528:H528"/>
     <mergeCell ref="A585:H585"/>
@@ -19138,6 +19130,11 @@
     <mergeCell ref="A353:H353"/>
     <mergeCell ref="A411:H411"/>
     <mergeCell ref="A463:H463"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A94:H94"/>
+    <mergeCell ref="A134:H134"/>
+    <mergeCell ref="I144:I147"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -19152,16 +19149,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -22502,16 +22499,16 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -24952,10 +24949,10 @@
       <c r="G1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="J1" s="1"/>
+      <c r="J1" s="3"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -25228,10 +25225,10 @@
       <c r="G11">
         <v>42659.163342900007</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -27005,10 +27002,10 @@
       <c r="H11" t="s">
         <v>258</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="I11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="3"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -27166,7 +27163,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="5" width="11.5" bestFit="1" customWidth="1"/>
@@ -27208,19 +27205,19 @@
       <c r="C2" t="s">
         <v>197</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>28355.0347050036</v>
       </c>
-      <c r="E2" s="2">
-        <f t="shared" ref="E2:E26" si="0">D2/IF(B2="MENSUAL",12,IF(B2="TRIMESTRAL",4,IF(B2="SEMESTRAL",2,1)))</f>
+      <c r="E2" s="1">
+        <f t="shared" ref="E2:E25" si="0">D2/IF(B2="MENSUAL",12,IF(B2="TRIMESTRAL",4,IF(B2="SEMESTRAL",2,1)))</f>
         <v>2362.9195587503</v>
       </c>
       <c r="G2" t="s">
         <v>244</v>
       </c>
       <c r="H2">
-        <f>SUMIF(C2:C26,"VIDA",E2:E26)</f>
-        <v>563907.97513739287</v>
+        <f>SUMIF(C2:C25,"VIDA",E2:E25)</f>
+        <v>561595.36778714287</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -27233,10 +27230,10 @@
       <c r="C3" t="s">
         <v>197</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>24718.650359059997</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <f t="shared" si="0"/>
         <v>12359.325179529998</v>
       </c>
@@ -27244,7 +27241,7 @@
         <v>246</v>
       </c>
       <c r="H3">
-        <f>SUMIF(C2:C26,"GMM",E2:E26)</f>
+        <f>SUMIF(C2:C25,"GMM",E2:E25)</f>
         <v>37128.26</v>
       </c>
     </row>
@@ -27258,10 +27255,10 @@
       <c r="C4" t="s">
         <v>197</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>96899.18338314</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <f t="shared" si="0"/>
         <v>96899.18338314</v>
       </c>
@@ -27269,7 +27266,7 @@
         <v>247</v>
       </c>
       <c r="H4">
-        <f>COUNTIF(C2:C26,"GMM")</f>
+        <f>COUNTIF(C2:C25,"GMM")</f>
         <v>5</v>
       </c>
     </row>
@@ -27283,10 +27280,10 @@
       <c r="C5" t="s">
         <v>197</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>66100.985070369992</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <f t="shared" si="0"/>
         <v>66100.985070369992</v>
       </c>
@@ -27294,8 +27291,8 @@
         <v>245</v>
       </c>
       <c r="H5">
-        <f>COUNTIF(C2:C26,"VIDA")</f>
-        <v>20</v>
+        <f>COUNTIF(C2:C25,"VIDA")</f>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -27308,10 +27305,10 @@
       <c r="C6" t="s">
         <v>197</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>33322.854766909993</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <f t="shared" si="0"/>
         <v>33322.854766909993</v>
       </c>
@@ -27326,10 +27323,10 @@
       <c r="C7" t="s">
         <v>197</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>73112.783475479999</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <f t="shared" si="0"/>
         <v>6092.7319562900002</v>
       </c>
@@ -27344,10 +27341,10 @@
       <c r="C8" t="s">
         <v>197</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>23580.417253862401</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <f t="shared" si="0"/>
         <v>1965.0347711552001</v>
       </c>
@@ -27362,10 +27359,10 @@
       <c r="C9" t="s">
         <v>194</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>65420.399999999994</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <f t="shared" si="0"/>
         <v>5451.7</v>
       </c>
@@ -27380,10 +27377,10 @@
       <c r="C10" t="s">
         <v>197</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>90033.454256679994</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <f t="shared" si="0"/>
         <v>90033.454256679994</v>
       </c>
@@ -27398,10 +27395,10 @@
       <c r="C11" t="s">
         <v>197</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>23527.39078944</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <f t="shared" si="0"/>
         <v>1960.61589912</v>
       </c>
@@ -27416,10 +27413,10 @@
       <c r="C12" t="s">
         <v>194</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>27662.28</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <f t="shared" si="0"/>
         <v>2305.19</v>
       </c>
@@ -27434,10 +27431,10 @@
       <c r="C13" t="s">
         <v>197</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>83019.199999999997</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <f t="shared" si="0"/>
         <v>83019.199999999997</v>
       </c>
@@ -27452,10 +27449,10 @@
       <c r="C14" t="s">
         <v>197</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>36338.399738128799</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <f t="shared" si="0"/>
         <v>3028.1999781773998</v>
       </c>
@@ -27470,10 +27467,10 @@
       <c r="C15" t="s">
         <v>197</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>58335.862101919993</v>
       </c>
-      <c r="E15" s="2">
+      <c r="E15" s="1">
         <f t="shared" si="0"/>
         <v>58335.862101919993</v>
       </c>
@@ -27488,10 +27485,10 @@
       <c r="C16" t="s">
         <v>197</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>28766.235240000005</v>
       </c>
-      <c r="E16" s="2">
+      <c r="E16" s="1">
         <f t="shared" si="0"/>
         <v>2397.1862700000006</v>
       </c>
@@ -27506,10 +27503,10 @@
       <c r="C17" t="s">
         <v>197</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>34327.825434270002</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="1">
         <f t="shared" si="0"/>
         <v>34327.825434270002</v>
       </c>
@@ -27524,10 +27521,10 @@
       <c r="C18" t="s">
         <v>197</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>29809.2060079</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="1">
         <f t="shared" si="0"/>
         <v>29809.2060079</v>
       </c>
@@ -27542,10 +27539,10 @@
       <c r="C19" t="s">
         <v>194</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>26627.46</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19" s="1">
         <f t="shared" si="0"/>
         <v>26627.46</v>
       </c>
@@ -27560,10 +27557,10 @@
       <c r="C20" t="s">
         <v>197</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>36672.004980719998</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="1">
         <f t="shared" si="0"/>
         <v>3056.0004150599998</v>
       </c>
@@ -27578,10 +27575,10 @@
       <c r="C21" t="s">
         <v>197</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>20910.710278080001</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="1">
         <f t="shared" si="0"/>
         <v>1742.55918984</v>
       </c>
@@ -27596,10 +27593,10 @@
       <c r="C22" t="s">
         <v>197</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="1">
         <v>36755.186497499999</v>
       </c>
-      <c r="E22" s="2">
+      <c r="E22" s="1">
         <f t="shared" si="0"/>
         <v>18377.593248749999</v>
       </c>
@@ -27614,10 +27611,10 @@
       <c r="C23" t="s">
         <v>194</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="1">
         <v>24314.639999999999</v>
       </c>
-      <c r="E23" s="2">
+      <c r="E23" s="1">
         <f t="shared" si="0"/>
         <v>2026.22</v>
       </c>
@@ -27632,46 +27629,28 @@
       <c r="C24" t="s">
         <v>197</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="1">
         <v>32809.260598559995</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="1">
         <f t="shared" si="0"/>
         <v>16404.630299279997</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B25" t="s">
         <v>199</v>
       </c>
       <c r="C25" t="s">
-        <v>197</v>
-      </c>
-      <c r="D25" s="2">
-        <v>27751.288203000007</v>
-      </c>
-      <c r="E25" s="2">
-        <f t="shared" si="0"/>
-        <v>2312.6073502500008</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>261</v>
-      </c>
-      <c r="B26" t="s">
-        <v>199</v>
-      </c>
-      <c r="C26" t="s">
         <v>194</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D25" s="1">
         <v>8612.2800000000007</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E25" s="1">
         <f t="shared" si="0"/>
         <v>717.69</v>
       </c>
@@ -27679,7 +27658,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H26" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:H24 A25:E25 F25:H26" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -27702,31 +27681,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="H1" t="s">
         <v>258</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>125</v>
       </c>
       <c r="J1" t="s">
@@ -27743,25 +27722,25 @@
       <c r="C2">
         <v>2</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>163000.16845350998</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
         <v>163000.16845350998</v>
       </c>
       <c r="H2" t="s">
         <v>258</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="J2" s="2">
+      <c r="J2" s="1">
         <v>563907.97513739299</v>
       </c>
     </row>
@@ -27775,22 +27754,22 @@
       <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>64137.031442170002</v>
       </c>
       <c r="E3">
         <v>0.5</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>26627.46</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="1">
         <v>90764.491442169994</v>
       </c>
       <c r="H3" t="s">
         <v>258</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>245</v>
       </c>
       <c r="J3">
@@ -27807,25 +27786,25 @@
       <c r="C4">
         <v>1</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>90033.454256679994</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" s="2">
-        <v>0</v>
-      </c>
-      <c r="G4" s="2">
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
         <v>90033.454256679994</v>
       </c>
       <c r="H4" t="s">
         <v>258</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="J4" s="2">
+      <c r="J4" s="1">
         <v>37128.26</v>
       </c>
     </row>
@@ -27839,22 +27818,22 @@
       <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>86047.399978177404</v>
       </c>
       <c r="E5">
         <v>0.5</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>2305.19</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="1">
         <v>88352.589978177406</v>
       </c>
       <c r="H5" t="s">
         <v>258</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>247</v>
       </c>
       <c r="J5">
@@ -27871,22 +27850,22 @@
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>58335.862101919993</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
-      <c r="F6" s="2">
-        <v>0</v>
-      </c>
-      <c r="G6" s="2">
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
         <v>58335.862101919993</v>
       </c>
       <c r="H6" t="s">
         <v>258</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>248</v>
       </c>
       <c r="J6">
@@ -27903,25 +27882,25 @@
       <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>33322.854766909993</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
-      <c r="F7" s="2">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2">
+      <c r="F7" s="1">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
         <v>33322.854766909993</v>
       </c>
       <c r="H7" t="s">
         <v>258</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="J7" s="2">
+      <c r="J7" s="1">
         <v>601036.23513739277</v>
       </c>
     </row>
@@ -27935,16 +27914,16 @@
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>18377.593248749999</v>
       </c>
       <c r="E8">
         <v>0.5</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>2026.22</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="1">
         <v>20403.813248750001</v>
       </c>
       <c r="H8" t="s">
@@ -27962,21 +27941,21 @@
         <v>170</v>
       </c>
       <c r="B9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>2</v>
-      </c>
-      <c r="D9" s="2">
-        <v>18717.237649529998</v>
+        <v>1</v>
+      </c>
+      <c r="D9" s="1">
+        <v>16404.630299279997</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
-      <c r="F9" s="2">
-        <v>0</v>
-      </c>
-      <c r="G9" s="2">
+      <c r="F9" s="1">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
         <v>18717.237649529998</v>
       </c>
       <c r="H9" t="s">
@@ -27999,16 +27978,16 @@
       <c r="C10">
         <v>2</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>14722.244738280298</v>
       </c>
       <c r="E10">
         <v>0</v>
       </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
         <v>14722.244738280298</v>
       </c>
       <c r="H10" t="s">
@@ -28031,22 +28010,22 @@
       <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>1965.0347711552001</v>
       </c>
       <c r="E11">
         <v>0.5</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>5451.7</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="1">
         <v>7416.7347711552002</v>
       </c>
       <c r="H11" t="s">
         <v>258</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I11" s="2" t="s">
         <v>56</v>
       </c>
       <c r="J11" t="s">
@@ -28063,26 +28042,26 @@
       <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>6092.7319562900002</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
-      <c r="F12" s="2">
-        <v>0</v>
-      </c>
-      <c r="G12" s="2">
+      <c r="F12" s="1">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1">
         <v>6092.7319562900002</v>
       </c>
       <c r="H12" t="s">
         <v>258</v>
       </c>
-      <c r="I12" s="3" t="s">
+      <c r="I12" s="2" t="s">
         <v>132</v>
       </c>
       <c r="J12" t="s">
-        <v>269</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
@@ -28095,22 +28074,22 @@
       <c r="C13">
         <v>2</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>4798.5596048999996</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
-      <c r="F13" s="2">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2">
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
         <v>4798.5596048999996</v>
       </c>
       <c r="H13" t="s">
         <v>258</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="I13" s="2" t="s">
         <v>134</v>
       </c>
       <c r="J13" t="s">
@@ -28127,22 +28106,22 @@
       <c r="C14">
         <v>1</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>2397.1862700000006</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
-      <c r="F14" s="2">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2">
+      <c r="F14" s="1">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1">
         <v>2397.1862700000006</v>
       </c>
       <c r="H14" t="s">
         <v>258</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="I14" s="2" t="s">
         <v>136</v>
       </c>
       <c r="J14" t="s">
@@ -28159,22 +28138,22 @@
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>1960.61589912</v>
       </c>
       <c r="E15">
         <v>0</v>
       </c>
-      <c r="F15" s="2">
-        <v>0</v>
-      </c>
-      <c r="G15" s="2">
+      <c r="F15" s="1">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
         <v>1960.61589912</v>
       </c>
       <c r="H15" t="s">
         <v>258</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="2" t="s">
         <v>137</v>
       </c>
       <c r="J15" t="s">
@@ -28197,27 +28176,27 @@
       <c r="E16">
         <v>0.5</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="1">
         <v>717.69</v>
       </c>
-      <c r="G16" s="2">
+      <c r="G16" s="1">
         <v>717.69</v>
       </c>
       <c r="H16" t="s">
         <v>258</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="I16" s="2" t="s">
         <v>138</v>
       </c>
       <c r="J16" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H17" t="s">
         <v>258</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="I17" s="2" t="s">
         <v>140</v>
       </c>
       <c r="J17" t="s">
@@ -28228,18 +28207,18 @@
       <c r="H18" t="s">
         <v>258</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="I18" s="2" t="s">
         <v>141</v>
       </c>
       <c r="J18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="8:10" x14ac:dyDescent="0.2">
       <c r="H19" t="s">
         <v>258</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="I19" s="2" t="s">
         <v>143</v>
       </c>
       <c r="J19" t="s">

</xml_diff>